<commit_message>
Adjusts economically retrofitted CCS to account for initial deployment; formula fixes; adds BAU economic CCS; ties into cash flows
</commit_message>
<xml_diff>
--- a/InputData/ccs/CCP/CO2 Capture Potentials.xlsx
+++ b/InputData/ccs/CCP/CO2 Capture Potentials.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\ccs\CCP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\ccs\CCP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28C2AF75-4449-4234-82F2-ED89CB505329}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E989DDD-D587-494A-AC19-566F1124067F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26775" yWindow="1005" windowWidth="25275" windowHeight="12525" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="CPPbES" sheetId="12" r:id="rId2"/>
-    <sheet name="CPPbI" sheetId="13" r:id="rId3"/>
-    <sheet name="CPPbHS" sheetId="15" r:id="rId4"/>
+    <sheet name="CPPbHS" sheetId="15" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="45">
   <si>
     <t>Source:</t>
   </si>
@@ -42,9 +41,6 @@
   </si>
   <si>
     <t>None</t>
-  </si>
-  <si>
-    <t>CPP CO2 Capture Potential by Industry</t>
   </si>
   <si>
     <t>CPP CO2 Capture Potential by Electricity Source</t>
@@ -202,87 +198,6 @@
     </r>
   </si>
   <si>
-    <t>energy related emissions</t>
-  </si>
-  <si>
-    <t>process emissions</t>
-  </si>
-  <si>
-    <t>agriculture and forestry 01T03</t>
-  </si>
-  <si>
-    <t>coal mining 05</t>
-  </si>
-  <si>
-    <t>oil and gas extraction 06</t>
-  </si>
-  <si>
-    <t>other mining and quarrying 07T08</t>
-  </si>
-  <si>
-    <t>food beverage and tobacco 10T12</t>
-  </si>
-  <si>
-    <t>textiles apparel and leather 13T15</t>
-  </si>
-  <si>
-    <t>wood products 16</t>
-  </si>
-  <si>
-    <t>pulp paper and printing 17T18</t>
-  </si>
-  <si>
-    <t>refined petroleum and coke 19</t>
-  </si>
-  <si>
-    <t>chemicals 20</t>
-  </si>
-  <si>
-    <t>rubber and plastic products 22</t>
-  </si>
-  <si>
-    <t>glass and glass products 231</t>
-  </si>
-  <si>
-    <t>cement and other nonmetallic minerals 239</t>
-  </si>
-  <si>
-    <t>iron and steel 241</t>
-  </si>
-  <si>
-    <t>other metals 242</t>
-  </si>
-  <si>
-    <t>metal products except machinery and vehicles 25</t>
-  </si>
-  <si>
-    <t>computers and electronics 26</t>
-  </si>
-  <si>
-    <t>appliances and electrical equipment 27</t>
-  </si>
-  <si>
-    <t>other machinery 28</t>
-  </si>
-  <si>
-    <t>road vehicles 29</t>
-  </si>
-  <si>
-    <t>nonroad vehicles 30</t>
-  </si>
-  <si>
-    <t>other manufacturing 31T33</t>
-  </si>
-  <si>
-    <t>energy pipelines and gas processing 352T353</t>
-  </si>
-  <si>
-    <t>water and waste 36T39</t>
-  </si>
-  <si>
-    <t>construction 41T43</t>
-  </si>
-  <si>
     <t>For industries, we assign 100% to all industries except mining, agriculture, construction, and water and waste, as the activities</t>
   </si>
   <si>
@@ -320,6 +235,9 @@
   </si>
   <si>
     <t>capture rate</t>
+  </si>
+  <si>
+    <t>CPP CO2 Capture Potential by Hydrogen Sector</t>
   </si>
 </sst>
 </file>
@@ -732,7 +650,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -750,22 +668,22 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -776,33 +694,33 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="2"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="2"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="2"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="2"/>
@@ -813,24 +731,24 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B22" s="6"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B23" s="6"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -852,12 +770,12 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -865,7 +783,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="B3">
         <v>0</v>
@@ -873,7 +791,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -881,7 +799,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -889,7 +807,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6">
         <v>0</v>
@@ -897,7 +815,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -905,7 +823,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -913,7 +831,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -921,7 +839,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -929,7 +847,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -937,7 +855,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -945,7 +863,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -953,7 +871,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14">
         <v>0</v>
@@ -961,7 +879,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -969,7 +887,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B16">
         <v>0</v>
@@ -977,7 +895,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -985,7 +903,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -993,7 +911,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="B19">
         <v>0.95</v>
@@ -1001,7 +919,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="B20">
         <v>0.95</v>
@@ -1009,7 +927,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>65</v>
+        <v>37</v>
       </c>
       <c r="B21">
         <v>0.95</v>
@@ -1017,7 +935,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="B22">
         <v>0.95</v>
@@ -1025,7 +943,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -1033,7 +951,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -1041,7 +959,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -1054,310 +972,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D5F30A2-728A-4F27-B64D-DBC772B5208E}">
-  <sheetPr>
-    <tabColor theme="3"/>
-  </sheetPr>
-  <dimension ref="A1:C26"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="45.42578125" customWidth="1"/>
-    <col min="2" max="2" width="24.7109375" customWidth="1"/>
-    <col min="3" max="3" width="25.85546875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>42</v>
-      </c>
-      <c r="B10">
-        <v>1</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11">
-        <v>1</v>
-      </c>
-      <c r="C11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>44</v>
-      </c>
-      <c r="B12">
-        <v>1</v>
-      </c>
-      <c r="C12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>45</v>
-      </c>
-      <c r="B13">
-        <v>1</v>
-      </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B14">
-        <v>1</v>
-      </c>
-      <c r="C14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>47</v>
-      </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
-      <c r="C15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>48</v>
-      </c>
-      <c r="B16">
-        <v>1</v>
-      </c>
-      <c r="C16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>49</v>
-      </c>
-      <c r="B17">
-        <v>1</v>
-      </c>
-      <c r="C17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>50</v>
-      </c>
-      <c r="B18">
-        <v>1</v>
-      </c>
-      <c r="C18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>51</v>
-      </c>
-      <c r="B19">
-        <v>1</v>
-      </c>
-      <c r="C19">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>52</v>
-      </c>
-      <c r="B20">
-        <v>1</v>
-      </c>
-      <c r="C20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>53</v>
-      </c>
-      <c r="B21">
-        <v>1</v>
-      </c>
-      <c r="C21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>54</v>
-      </c>
-      <c r="B22">
-        <v>1</v>
-      </c>
-      <c r="C22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>55</v>
-      </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
-      <c r="C23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>56</v>
-      </c>
-      <c r="B24">
-        <v>1</v>
-      </c>
-      <c r="C24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>57</v>
-      </c>
-      <c r="B25">
-        <v>0</v>
-      </c>
-      <c r="C25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>58</v>
-      </c>
-      <c r="B26">
-        <v>0</v>
-      </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D48B9D0-7C8A-4023-B3D1-3CE3C9AF0583}">
   <sheetPr>
     <tabColor theme="3"/>
@@ -1372,15 +986,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B1" t="s">
-        <v>71</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>42</v>
       </c>
       <c r="B2">
         <v>0.85</v>

</xml_diff>